<commit_message>
Refactor core workflow handling
</commit_message>
<xml_diff>
--- a/reports/tigrbl_tests_matrices.xlsx
+++ b/reports/tigrbl_tests_matrices.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <sheets>
     <sheet name="Legend" sheetId="1" state="visible" r:id="rId1"/>
@@ -10,7 +10,7 @@
     <sheet name="P1 Linked" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="P2 Core" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="P3 Examples" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="P4 Edge" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Legacy Edge" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="P0 op_ctx Map" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="New ADRs" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="New SPECs" sheetId="11" state="visible" r:id="rId11"/>
@@ -44916,228 +44916,485 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:V4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="47" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="56" customWidth="1"/>
+    <col min="11" max="11" width="70" customWidth="1"/>
+    <col min="12" max="12" width="90" customWidth="1"/>
+    <col min="13" max="13" width="38" customWidth="1"/>
+    <col min="14" max="14" width="80" customWidth="1"/>
+    <col min="15" max="15" width="50" customWidth="1"/>
+    <col min="16" max="16" width="90" customWidth="1"/>
+    <col min="17" max="17" width="48" customWidth="1"/>
+    <col min="18" max="18" width="70" customWidth="1"/>
+    <col min="19" max="19" width="48" customWidth="1"/>
+    <col min="20" max="20" width="70" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="80" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>concern_bucket</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>primary_concern</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>secondary_concerns</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>test_path</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>test_file</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>marker</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>function</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>adr</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>spec</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>feature</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>feature_linked</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>priority_precedence</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>traceability_status</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>candidate_rationale</t>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>ssot_registered</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>test_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>feature_ids</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>feature_titles</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>spec_ids</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t>spec_titles</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t>adr_ids</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t>adr_titles</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t>claim_ids</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t>claim_titles</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t>evidence_ids</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr" s="1">
+        <is>
+          <t>evidence_titles</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr" s="1">
+        <is>
+          <t>link_status</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr" s="1">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>legacy-package-edge</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pre-tx dependency execution</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>security dependency ordering; failure aborts handler execution</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pkgs/core/tigrbl_tests/tests/test_secdeps_execute_in_pre_tx.py</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>tests/test_secdeps_execute_in_pre_tx.py</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>asyncio</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>tests-root</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>secdeps execute in pre tx</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>candidate:ADR-1011; candidate:ADR-1032; candidate:ADR-1037</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>candidate:SPEC-2012</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>tst:pkgs-core-tigrbl_tests-tests-test_secdeps_execute_in_pre_tx.py</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>feat:pre-tx-dependency-execution-001; feat:pre-tx-security-dependency-execution-001; feat:anon-access-projection-001; feat:anon-access-rest-status-parity-001; feat:apikey-security-dependency-001; feat:auth-failure-projection-parity-001; feat:error-envelope-structure-parity-001; feat:error-parity-response-structure-001; feat:httpbasic-security-dependency-001; feat:httpbearer-security-dependency-001; feat:jsonrpc-batch-framing-001; feat:mutualtls-security-dependency-001; feat:oauth2-security-dependency-001; feat:openidconnect-security-dependency-001; feat:rest-create-success-status-001; feat:security-concrete-dependency-helper-001; feat:validation-failure-projection-parity-001</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>feat:pre-tx-dependency-execution-001 (Pre-TX dependency execution); feat:pre-tx-security-dependency-execution-001 (Pre-TX security dependency execution); feat:anon-access-projection-001 (Anonymous access projection); feat:anon-access-rest-status-parity-001 (Anonymous access and REST create status parity); feat:apikey-security-dependency-001 (APIKey security dependency); feat:auth-failure-projection-parity-001 (Authorization failure projection parity); feat:error-envelope-structure-parity-001 (Error envelope structure parity); feat:error-parity-response-structure-001 (Error parity, validation parity, and response structure); feat:httpbasic-security-dependency-001 (HTTPBasic security dependency); feat:httpbearer-security-dependency-001 (HTTPBearer security dependency); feat:jsonrpc-batch-framing-001 (JSON-RPC batch framing); feat:mutualtls-security-dependency-001 (MutualTLS security dependency); feat:oauth2-security-dependency-001 (OAuth2 security dependency); feat:openidconnect-security-dependency-001 (OpenIdConnect security dependency); feat:rest-create-success-status-001 (REST create success status projection); feat:security-concrete-dependency-helper-001 (Security concrete dependency helper); feat:validation-failure-projection-parity-001 (Validation failure projection parity)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>spc:2074; spc:2044; spc:2012; spc:2080; spc:2020</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>spc:2074 (Pre-TX dependency execution contract); spc:2044 (Concrete dependency helper surface); spc:2012 (Status, Auth, and Error Parity); spc:2080 (Documentation runtime parity contract); spc:2020 (Operator-surface framing and multipart semantics)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>adr:1078; adr:1032; adr:1011; adr:1037; adr:1014; adr:1080; adr:1041</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>adr:1078 (Pre-TX dependency execution boundary); adr:1032 (Status, Auth, and Error Projections Derive from Canonical Outcomes); adr:1011 (ADR-0011 â€” Security Deps and Deps Ordering); adr:1037 (OAS 3.1 security-scheme-first architecture); adr:1014 (REST and JSON-RPC Semantic Parity); adr:1080 (Documentation support surface partitioning); adr:1041 (Operator-surface boundary)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>clm:pre-tx-dependency-execution-contract-001</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>clm:pre-tx-dependency-execution-contract-001 (Pre-TX dependencies execute before transaction and handler)</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>evd:pre-tx-dependency-execution-pytest</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>evd:pre-tx-dependency-execution-pytest (Pre-TX dependency execution pytest)</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>fully_linked</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Primary: pre-TX dependency execution. Secondary: security deps run before extra deps; dependency failure prevents handler execution.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>legacy-package-edge</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>governed ORM alias compatibility</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>tigrbl.orm.mixins projection; Bootstrappable compatibility export</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pkgs/core/tigrbl_tests/tigrbl_tests/tests/test_orm_alias_exports.py</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>tigrbl_tests/tests/test_orm_alias_exports.py</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>package-smoke</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>orm alias exports</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>tst:pkgs-core-tigrbl_tests-tigrbl_tests-tests-test_orm_alias_exports.py</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>feat:governed-module-alias-compatibility-001; feat:orm-alias-export-compatibility-001; feat:orm-mixins-alias-compatibility-001; feat:bootstrappable-table-mixin-001; feat:tigrbl-test-suite-coverage-intake-001</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>feat:governed-module-alias-compatibility-001 (Governed module alias compatibility); feat:orm-alias-export-compatibility-001 (tigrbl.orm alias export compatibility); feat:orm-mixins-alias-compatibility-001 (tigrbl.orm.mixins alias compatibility); feat:bootstrappable-table-mixin-001 (Bootstrappable table mixin); feat:tigrbl-test-suite-coverage-intake-001 (Tigrbl test suite coverage intake)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>spc:2025; spc:2038; spc:2039</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>spc:2025 (tigrbl_core._spec Private and Public Export Surface); spc:2038 (Table mixins surface); spc:2039 (Bootstrappable table ORM mixin defaults and seeding)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>adr:1003; adr:1052; adr:1056; adr:1053; adr:1018; adr:1055</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>adr:1003 (ADR-0003 â€” Spec-First Authoritative Spec Layer); adr:1052 (tigrbl_core._spec Layer Nature and Authority); adr:1056 (Table mixins and bootstrappable defaults); adr:1053 (tigrbl_base Layer Nature and Authority); adr:1018 (ADR-0018 â€” Shortcuts and Aliases Expand to Canonical Forms); adr:1055 (DDL surface ownership and initialization boundary)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>clm:orm-alias-export-compatibility-001</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>clm:orm-alias-export-compatibility-001 (ORM alias exports remain import-compatible)</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>evd:orm-alias-export-compatibility-pytest</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>evd:orm-alias-export-compatibility-pytest (ORM alias export compatibility pytest)</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>fully_linked</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Primary: governed import alias compatibility. Secondary: Bootstrappable must remain available through tigrbl.orm.mixins.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>legacy-package-edge</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AppSpec/RouterSpec typed composition</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RouterSpec-owned tables; TableSpec.model_ref; nested ColumnSpec metadata</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pkgs/core/tigrbl_tests/v4/tests/spec/test_master_app_spec_surface.py</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>v4/tests/spec/test_master_app_spec_surface.py</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>v4-spec</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>spec / master app spec surface</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>tst:pkgs-core-tigrbl_tests-v4-tests-spec-test_master_app_spec_surface.py</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>feat:appspec-routerspec-composition-001; feat:appspec-contract-001; feat:routerspec-contract-001; feat:tablespec-contract-001; feat:columnspec-contract-001; feat:storagespec-contract-001; feat:fieldspec-contract-001; feat:iospec-contract-001; feat:foreignkeyspec-contract-001; feat:opspec-contract-001; feat:responsespec-contract-001; feat:tigrbl-test-suite-coverage-intake-001</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>feat:appspec-routerspec-composition-001 (AppSpec and RouterSpec composition); feat:appspec-contract-001 (AppSpec contract); feat:routerspec-contract-001 (RouterSpec contract); feat:tablespec-contract-001 (TableSpec contract); feat:columnspec-contract-001 (ColumnSpec contract); feat:storagespec-contract-001 (StorageSpec contract); feat:fieldspec-contract-001 (FieldSpec contract); feat:iospec-contract-001 (IOSpec contract); feat:foreignkeyspec-contract-001 (ForeignKeySpec contract); feat:opspec-contract-001 (OpSpec contract); feat:responsespec-contract-001 (ResponseSpec contract); feat:tigrbl-test-suite-coverage-intake-001 (Tigrbl test suite coverage intake)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>spc:1000; spc:2025; spc:2064; spc:2065; spc:2068</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>spc:1000 (AppSpec and RouterSpec composition contract); spc:2025 (tigrbl_core._spec Private and Public Export Surface); spc:2064 (Op alias and target resolution contract); spc:2065 (Default OLTP op projection contract); spc:2068 (OpSpec materialization effects contract)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>adr:1003; adr:1052; adr:1001; adr:1013; adr:1018; adr:1072; adr:1014; adr:1047; adr:1051; adr:1074; adr:1075</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>adr:1003 (ADR-0003 â€” Spec-First Authoritative Spec Layer); adr:1052 (tigrbl_core._spec Layer Nature and Authority); adr:1001 (ADR-0001 â€” One Semantic Op Model); adr:1013 (ADR-0013 â€” Default Canonical OLTP Ops); adr:1018 (ADR-0018 â€” Shortcuts and Aliases Expand to Canonical Forms); adr:1072 (Alias versus target resolution boundary); adr:1014 (REST and JSON-RPC Semantic Parity); adr:1047 (ADR-1047 - KernelPlan-Owned Transport Dispatch); adr:1051 (Canonical Path-Keyed Transport Routing Tuple); adr:1074 (Default op collision and capability precedence); adr:1075 (OpSpec materialization side-effect boundary)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>clm:appspec-routerspec-composition-contract-001</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>clm:appspec-routerspec-composition-contract-001 (AppSpec and RouterSpec nested composition remains typed)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>evd:appspec-routerspec-composition-pytest</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>evd:appspec-routerspec-composition-pytest (AppSpec RouterSpec composition pytest)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>fully_linked</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Primary: AppSpec.routers accepts RouterSpec with router-owned TableSpec entries. Secondary: nested response/op/storage/field/io/fk metadata remains typed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:V4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>